<commit_message>
workflow: finalize xlsx-only cleanup
</commit_message>
<xml_diff>
--- a/know-all/outputs/20260322_咖啡/01_审核稿.xlsx
+++ b/know-all/outputs/20260322_咖啡/01_审核稿.xlsx
@@ -39,6 +39,7 @@
     </font>
     <font>
       <name val="Microsoft YaHei"/>
+      <color rgb="00222222"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -72,20 +73,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -456,13 +456,13 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="54" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
+    <col width="54" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -471,45 +471,40 @@
           <t>专题信息</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>专题</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>咖啡</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>专题</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>咖啡</t>
-        </is>
-      </c>
-    </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>这份本地表格是当前审核阶段唯一 source of truth。</t>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>本地审核表格是审核阶段唯一 source of truth。只有在用户明确确认后，才允许进入出图。</t>
         </is>
       </c>
     </row>
@@ -520,7 +515,7 @@
           <t>标题</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>每日闲聊语料库｜咖啡：很多人天天喝，但这5件事一直没弄明白☕</t>
         </is>
@@ -535,24 +530,24 @@
       </c>
     </row>
     <row r="9" ht="24" customHeight="1">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>主标题</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>很多人喝咖啡，但没真搞懂咖啡</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>副标题</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>从酸苦到咖啡因，这几件事最容易想当然</t>
         </is>
@@ -560,454 +555,417 @@
     </row>
     <row r="11" ht="24" customHeight="1"/>
     <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>封面列点</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>mark_raw</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>mark_render</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>文本</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>☕</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>苦</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>苦不等于更浓</t>
         </is>
       </c>
     </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>🍋</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>酸</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>酸味不一定坏了</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>🌑</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>深</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>深烘不一定更提神</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>✨</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>豆</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>豆子发油未必更好</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="78" customHeight="1">
-      <c r="A18" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>🧊</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>冰</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>冰美式也可能很顶</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="78" customHeight="1"/>
-    <row r="20" ht="78" customHeight="1">
+    <row r="19" ht="24" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1">
       <c r="A20" s="1" t="inlineStr">
         <is>
           <t>知识卡</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="78" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="21" ht="24" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>卡片ID</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>标题</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>mark_raw</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>mark_render</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>正文1</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F22" s="4" t="inlineStr">
         <is>
           <t>正文2</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>正文3</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>正文4</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="78" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>苦不等于更浓 ☕</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>☕</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>咖</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>很多人喝到一杯特别苦的咖啡，第一反应就是：这杯真浓。这个判断很常见，但其实“苦”和“浓”不是一回事。</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>咖啡的苦味，跟烘焙深浅、萃取时间、研磨粗细、水温这些因素都有关。萃过头了会苦，深烘豆本身也更容易往苦感走，但这不等于它的风味就更厚、更有层次。所谓“浓”，更接近咖啡液里可溶物的整体浓度和口感强度，不是舌头先尝到一点苦就能直接下结论。</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>所以有些咖啡喝起来很苦，其实只是萃取不太对；反过来，有些做得好的咖啡并不苦得吓人，但香气、甜感和厚度都很完整。苦只是其中一个味觉信号，不是整杯咖啡质量的总答案。</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="n"/>
-    </row>
-    <row r="23" ht="78" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="23" ht="92" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>酸味不一定坏了 🍋</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>🍋</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>酸</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>不少平时喝惯深烘或速溶的人，第一次喝到明显发酸的咖啡时，都会怀疑：这豆子是不是放坏了？</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>但咖啡里的“酸”，很多时候是正常风味的一部分。尤其浅烘豆，更容易保留果酸、花香和比较亮的风味，喝起来会有柑橘、莓果、青苹果这一类感觉。真正坏掉的酸，通常不是清亮的果酸，而是发闷、发馊、让人不舒服的那种酸败感。</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>也就是说，咖啡里的酸不能一概当成缺点。很多精品咖啡恰恰是靠这点酸把层次撑起来的。怕酸可以选风味更稳一点的豆子，但不能把“有酸感”和“坏了”直接画等号。</t>
         </is>
       </c>
-      <c r="H23" s="5" t="n"/>
-    </row>
-    <row r="24" ht="78" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="H23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="92" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>深烘不一定更提神 🌑</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>🌑</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>深</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>很多人会顺手觉得：颜色越深、味道越重的咖啡，应该越提神。这个印象很容易成立，因为深烘喝起来确实更“有存在感”。</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>但提神主要还是看咖啡因，不是看味道冲不冲。烘得深，更多是把风味往焦糖、坚果、烟熏这一边带，不是自动把咖啡因往上拉。真正影响你一杯喝下去有多顶的，往往是豆子本身、粉水比、萃取方式和你实际喝进去多少，而不是颜色看着有多黑。</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>所以深烘给人的“猛”，很多时候是味觉上的猛，不一定等于生理上的更提神。要判断一杯咖啡到底顶不顶，不能只凭它喝起来重不重。</t>
         </is>
       </c>
-      <c r="H24" s="5" t="n"/>
-    </row>
-    <row r="25" ht="78" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="H24" s="3" t="n"/>
+    </row>
+    <row r="25" ht="92" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>豆子发油未必更好 ✨</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>✨</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>豆</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>很多人看到咖啡豆表面亮亮油油的，会下意识觉得：这豆子状态不错，看着就高级。</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>但豆子表面出油，很多时候只是烘得更深，或者放了一段时间以后内部油脂慢慢跑到了表面。它说明的是烘焙程度和保存状态，不直接说明豆子品质更高。尤其如果一袋豆子放久了，表面越来越油，香气却在往下掉，那这个“油亮”反而未必是好消息。</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>所以咖啡豆看起来发不发油，不能直接拿来判断好坏。新鲜、保存得当、风味干净，往往比“表面很亮”更重要。</t>
         </is>
       </c>
-      <c r="H25" s="5" t="n"/>
-    </row>
-    <row r="26" ht="78" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="H25" s="3" t="n"/>
+    </row>
+    <row r="26" ht="92" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>冰美式也可能很顶 🧊</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>🧊</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>冰</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>很多人会把冰美式理解成一种“看起来最轻”的咖啡，觉得它颜色淡、没有奶、又加了冰，应该没那么刺激。</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>但一杯冰美式到底顶不顶，关键看里面放了几份浓缩。门店做法一旦不同，咖啡因差别就会很明显。有的杯子看着清清淡淡，其实底下塞了双份甚至更多浓缩；再加上它喝起来很快，没什么负担感，反而容易在短时间里灌下去更多。</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>所以冰美式“轻”很多时候只是视觉和口感上的轻，不一定等于咖啡因就低。尤其平时空腹、喝得快、又对咖啡因比较敏感的人，最容易被这种外表骗到。</t>
         </is>
       </c>
-      <c r="H26" s="5" t="n"/>
-    </row>
-    <row r="27" ht="78" customHeight="1"/>
-    <row r="28" ht="78" customHeight="1"/>
-    <row r="29" ht="78" customHeight="1"/>
-    <row r="30" ht="78" customHeight="1">
+      <c r="H26" s="3" t="n"/>
+    </row>
+    <row r="27" ht="92" customHeight="1"/>
+    <row r="28" ht="92" customHeight="1"/>
+    <row r="29" ht="24" customHeight="1"/>
+    <row r="30" ht="24" customHeight="1">
       <c r="A30" s="1" t="inlineStr">
         <is>
           <t>#话题</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="78" customHeight="1">
+    <row r="31" ht="24" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
           <t>话题</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="78" customHeight="1">
-      <c r="A32" t="inlineStr">
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>#咖啡知识</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="78" customHeight="1">
-      <c r="A33" t="inlineStr">
+    <row r="33" ht="24" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>#咖啡日常</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="78" customHeight="1">
-      <c r="A34" t="inlineStr">
+    <row r="34" ht="24" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>#咖啡入门</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="78" customHeight="1">
-      <c r="A35" t="inlineStr">
+    <row r="35" ht="24" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>#生活常识</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="78" customHeight="1">
-      <c r="A36" t="inlineStr">
+    <row r="36" ht="24" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>#涨知识</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="78" customHeight="1">
-      <c r="A37" t="inlineStr">
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>#每日闲聊语料库</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="78" customHeight="1"/>
-    <row r="39" ht="78" customHeight="1"/>
+    <row r="38" ht="24" customHeight="1"/>
+    <row r="39" ht="24" customHeight="1"/>
     <row r="40" ht="48" customHeight="1">
       <c r="A40" s="1" t="inlineStr">
         <is>
           <t>确认说明</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>请直接修改这份本地表格。只有在明确说“文稿无误”或“可以出图”后，才允许进入出图阶段。</t>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>请直接修改这份本地审核表格。只有在明确说“文稿无误”或“可以出图”后，才允许进入图片阶段。</t>
         </is>
       </c>
     </row>

</xml_diff>